<commit_message>
upgrade features and fix some bugs
</commit_message>
<xml_diff>
--- a/Templates/ComplexReportTemplate.xlsx
+++ b/Templates/ComplexReportTemplate.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Бахытжан\0. Табель по программам\0. Трудозатраты-хронометраж\MissionTime\Templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19440" windowHeight="11700"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19440" windowHeight="11700" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Прил.4 часть 1" sheetId="5" r:id="rId1"/>
     <sheet name="Прил.4 часть 2" sheetId="6" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="144525" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t xml:space="preserve">Наименование работы (услуги): </t>
   </si>
@@ -115,11 +120,14 @@
   <si>
     <t>Таблица учета трудозатрат</t>
   </si>
+  <si>
+    <t>Филиал АО "ЦЭНКИ" - Космический центр "Южный"</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="[$-419]d\ mmm;@"/>
@@ -537,7 +545,7 @@
     </a:clrScheme>
     <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -572,7 +580,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -749,7 +757,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -810,7 +818,9 @@
         <v>2</v>
       </c>
       <c r="B4" s="27"/>
-      <c r="C4" s="25"/>
+      <c r="C4" s="25" t="s">
+        <v>19</v>
+      </c>
       <c r="D4" s="25"/>
       <c r="E4" s="25"/>
       <c r="F4" s="25"/>
@@ -1059,7 +1069,9 @@
         <v>2</v>
       </c>
       <c r="B6" s="27"/>
-      <c r="C6" s="25"/>
+      <c r="C6" s="25" t="s">
+        <v>19</v>
+      </c>
       <c r="D6" s="25"/>
       <c r="E6" s="25"/>
       <c r="F6" s="25"/>

</xml_diff>